<commit_message>
simpler and more efficient homotopy with parameter gamma, support for multiple precision, faster search of duplicates
</commit_message>
<xml_diff>
--- a/Comparison_polynomial_RMEP.xlsx
+++ b/Comparison_polynomial_RMEP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\MEP\RMEP_homotopy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1299C9C6-ECFB-49B2-B792-63CB552D0344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21136CF9-9A8A-4958-BC24-0F0EABAECE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21936" yWindow="636" windowWidth="22176" windowHeight="17028" xr2:uid="{7D2D116B-6D63-4BF8-9BBB-ECD7956D1860}"/>
+    <workbookView xWindow="19140" yWindow="624" windowWidth="25860" windowHeight="17028" xr2:uid="{7D2D116B-6D63-4BF8-9BBB-ECD7956D1860}"/>
   </bookViews>
   <sheets>
     <sheet name="All data" sheetId="1" r:id="rId1"/>
@@ -760,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E596BE4F-61BA-409F-8651-028AAF812182}">
-  <dimension ref="A1:V141"/>
+  <dimension ref="A1:V142"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
@@ -4903,49 +4903,37 @@
         <v>3</v>
       </c>
       <c r="B77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C77">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D77">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E77">
         <v>0</v>
       </c>
       <c r="F77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G77">
-        <v>1458</v>
+        <v>2835</v>
       </c>
       <c r="H77" s="8">
-        <v>5.8984910836762688E-2</v>
+        <v>4.3099999999999999E-2</v>
       </c>
       <c r="I77" s="10">
-        <v>37.772519433013265</v>
-      </c>
-      <c r="J77" s="16">
-        <v>4.7204666666666667E-3</v>
+        <v>61.473999999999997</v>
       </c>
       <c r="K77" s="16">
-        <v>11.113312899999999</v>
+        <v>22.348199999999999</v>
       </c>
       <c r="L77" s="21">
-        <v>2.162323697391369E-14</v>
+        <v>3.4300000000000003E-14</v>
       </c>
       <c r="M77" s="21">
-        <v>3.3125786688416323E-16</v>
-      </c>
-      <c r="Q77" s="16">
-        <v>122.30894290000001</v>
-      </c>
-      <c r="R77" s="23">
-        <v>4.3606464890911999E-13</v>
-      </c>
-      <c r="S77" s="23">
-        <v>5.7434796010409036E-15</v>
+        <v>2.5000000000000002E-16</v>
       </c>
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.3">
@@ -4956,87 +4944,87 @@
         <v>5</v>
       </c>
       <c r="C78">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D78">
+        <v>3</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
         <v>1</v>
       </c>
-      <c r="E78">
-        <v>0</v>
-      </c>
-      <c r="F78">
-        <v>0</v>
-      </c>
       <c r="G78">
-        <v>5103</v>
+        <v>1458</v>
       </c>
       <c r="H78" s="8">
-        <v>6.8979031941994909E-2</v>
+        <v>5.8984910836762688E-2</v>
       </c>
       <c r="I78" s="10">
-        <v>39.8432294728591</v>
+        <v>37.772519433013265</v>
       </c>
       <c r="J78" s="16">
-        <v>1.4519900000000001E-2</v>
+        <v>4.7204666666666667E-3</v>
       </c>
       <c r="K78" s="16">
-        <v>48.186458100000003</v>
+        <v>11.113312899999999</v>
       </c>
       <c r="L78" s="21">
-        <v>1.2265086244831076E-13</v>
+        <v>2.162323697391369E-14</v>
       </c>
       <c r="M78" s="21">
-        <v>3.0241030583310743E-16</v>
+        <v>3.3125786688416323E-16</v>
+      </c>
+      <c r="Q78" s="16">
+        <v>122.30894290000001</v>
+      </c>
+      <c r="R78" s="23">
+        <v>4.3606464890911999E-13</v>
+      </c>
+      <c r="S78" s="23">
+        <v>5.7434796010409036E-15</v>
       </c>
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B79">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C79">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D79">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E79">
         <v>0</v>
       </c>
       <c r="F79">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>48</v>
+        <v>5103</v>
       </c>
       <c r="H79" s="8">
-        <v>2.4999999999999998E-2</v>
+        <v>6.8979031941994909E-2</v>
       </c>
       <c r="I79" s="10">
-        <v>35.091666666666661</v>
+        <v>39.8432294728591</v>
       </c>
       <c r="J79" s="16">
-        <v>6.6166E-4</v>
+        <v>1.4519900000000001E-2</v>
       </c>
       <c r="K79" s="16">
-        <v>0.20406301999999998</v>
+        <v>48.186458100000003</v>
       </c>
       <c r="L79" s="21">
-        <v>5.1636162701444704E-15</v>
+        <v>1.2265086244831076E-13</v>
       </c>
       <c r="M79" s="21">
-        <v>2.4050541761169982E-16</v>
-      </c>
-      <c r="Q79" s="16">
-        <v>5.1319119999999996E-2</v>
-      </c>
-      <c r="R79" s="23">
-        <v>1.9039088267757576E-14</v>
-      </c>
-      <c r="S79" s="23">
-        <v>1.9803021753882212E-15</v>
+        <v>3.0241030583310743E-16</v>
       </c>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.3">
@@ -5047,7 +5035,7 @@
         <v>2</v>
       </c>
       <c r="C80">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D80">
         <v>5</v>
@@ -5059,34 +5047,34 @@
         <v>5</v>
       </c>
       <c r="G80">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="H80" s="8">
         <v>2.4999999999999998E-2</v>
       </c>
       <c r="I80" s="10">
-        <v>35.543750000000003</v>
+        <v>35.091666666666661</v>
       </c>
       <c r="J80" s="16">
-        <v>8.9022000000000005E-4</v>
+        <v>6.6166E-4</v>
       </c>
       <c r="K80" s="16">
-        <v>0.35155676000000002</v>
+        <v>0.20406301999999998</v>
       </c>
       <c r="L80" s="21">
-        <v>6.6044339903193766E-15</v>
+        <v>5.1636162701444704E-15</v>
       </c>
       <c r="M80" s="21">
-        <v>2.0503553178939857E-16</v>
+        <v>2.4050541761169982E-16</v>
       </c>
       <c r="Q80" s="16">
-        <v>0.1038462</v>
+        <v>5.1319119999999996E-2</v>
       </c>
       <c r="R80" s="23">
-        <v>3.1544251439102089E-14</v>
+        <v>1.9039088267757576E-14</v>
       </c>
       <c r="S80" s="23">
-        <v>2.5974700552963143E-15</v>
+        <v>1.9803021753882212E-15</v>
       </c>
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.3">
@@ -5097,7 +5085,7 @@
         <v>2</v>
       </c>
       <c r="C81">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D81">
         <v>5</v>
@@ -5109,34 +5097,34 @@
         <v>5</v>
       </c>
       <c r="G81">
-        <v>160</v>
+        <v>96</v>
       </c>
       <c r="H81" s="8">
-        <v>1.7499999999999998E-2</v>
+        <v>2.4999999999999998E-2</v>
       </c>
       <c r="I81" s="10">
-        <v>37.651250000000005</v>
+        <v>35.543750000000003</v>
       </c>
       <c r="J81" s="16">
-        <v>1.12224E-3</v>
+        <v>8.9022000000000005E-4</v>
       </c>
       <c r="K81" s="16">
-        <v>0.63653746</v>
+        <v>0.35155676000000002</v>
       </c>
       <c r="L81" s="21">
-        <v>8.3112832032632516E-15</v>
+        <v>6.6044339903193766E-15</v>
       </c>
       <c r="M81" s="21">
-        <v>1.9875401159569674E-16</v>
+        <v>2.0503553178939857E-16</v>
       </c>
       <c r="Q81" s="16">
-        <v>0.20346367999999998</v>
+        <v>0.1038462</v>
       </c>
       <c r="R81" s="23">
-        <v>9.778811515855743E-13</v>
+        <v>3.1544251439102089E-14</v>
       </c>
       <c r="S81" s="23">
-        <v>2.2822300132756392E-14</v>
+        <v>2.5974700552963143E-15</v>
       </c>
     </row>
     <row r="82" spans="1:19" x14ac:dyDescent="0.3">
@@ -5147,7 +5135,7 @@
         <v>2</v>
       </c>
       <c r="C82">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D82">
         <v>5</v>
@@ -5159,34 +5147,34 @@
         <v>5</v>
       </c>
       <c r="G82">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="H82" s="8">
-        <v>2.5000000000000001E-2</v>
+        <v>1.7499999999999998E-2</v>
       </c>
       <c r="I82" s="10">
-        <v>39.858333333333334</v>
+        <v>37.651250000000005</v>
       </c>
       <c r="J82" s="16">
-        <v>1.5599599999999998E-3</v>
+        <v>1.12224E-3</v>
       </c>
       <c r="K82" s="16">
-        <v>1.0186321599999999</v>
+        <v>0.63653746</v>
       </c>
       <c r="L82" s="21">
-        <v>8.0165326312548139E-15</v>
+        <v>8.3112832032632516E-15</v>
       </c>
       <c r="M82" s="21">
-        <v>1.9164943387905609E-16</v>
+        <v>1.9875401159569674E-16</v>
       </c>
       <c r="Q82" s="16">
-        <v>0.41042536000000007</v>
+        <v>0.20346367999999998</v>
       </c>
       <c r="R82" s="23">
-        <v>1.8151501146785406E-13</v>
+        <v>9.778811515855743E-13</v>
       </c>
       <c r="S82" s="23">
-        <v>3.5174345616668639E-15</v>
+        <v>2.2822300132756392E-14</v>
       </c>
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.3">
@@ -5197,7 +5185,7 @@
         <v>2</v>
       </c>
       <c r="C83">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D83">
         <v>5</v>
@@ -5209,34 +5197,34 @@
         <v>5</v>
       </c>
       <c r="G83">
-        <v>336</v>
+        <v>240</v>
       </c>
       <c r="H83" s="8">
-        <v>1.6666666666666666E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="I83" s="10">
-        <v>41.69583333333334</v>
+        <v>39.858333333333334</v>
       </c>
       <c r="J83" s="16">
-        <v>1.9404399999999999E-3</v>
+        <v>1.5599599999999998E-3</v>
       </c>
       <c r="K83" s="16">
-        <v>1.5951258799999999</v>
+        <v>1.0186321599999999</v>
       </c>
       <c r="L83" s="21">
-        <v>8.2164339524242991E-15</v>
+        <v>8.0165326312548139E-15</v>
       </c>
       <c r="M83" s="21">
-        <v>1.8189827594694064E-16</v>
+        <v>1.9164943387905609E-16</v>
       </c>
       <c r="Q83" s="16">
-        <v>0.86774325999999991</v>
+        <v>0.41042536000000007</v>
       </c>
       <c r="R83" s="23">
-        <v>1.9036289092995512E-12</v>
+        <v>1.8151501146785406E-13</v>
       </c>
       <c r="S83" s="23">
-        <v>2.451769638850862E-14</v>
+        <v>3.5174345616668639E-15</v>
       </c>
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.3">
@@ -5247,7 +5235,7 @@
         <v>2</v>
       </c>
       <c r="C84">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D84">
         <v>5</v>
@@ -5259,34 +5247,34 @@
         <v>5</v>
       </c>
       <c r="G84">
-        <v>448</v>
+        <v>336</v>
       </c>
       <c r="H84" s="8">
-        <v>1.9642857142857146E-2</v>
+        <v>1.6666666666666666E-2</v>
       </c>
       <c r="I84" s="10">
-        <v>42.666964285714279</v>
+        <v>41.69583333333334</v>
       </c>
       <c r="J84" s="16">
-        <v>2.43888E-3</v>
+        <v>1.9404399999999999E-3</v>
       </c>
       <c r="K84" s="16">
-        <v>2.1699046600000003</v>
+        <v>1.5951258799999999</v>
       </c>
       <c r="L84" s="21">
-        <v>8.0746483171160317E-15</v>
+        <v>8.2164339524242991E-15</v>
       </c>
       <c r="M84" s="21">
-        <v>1.8361153524691382E-16</v>
+        <v>1.8189827594694064E-16</v>
       </c>
       <c r="Q84" s="16">
-        <v>1.41559104</v>
+        <v>0.86774325999999991</v>
       </c>
       <c r="R84" s="23">
-        <v>7.8049497441862349E-11</v>
+        <v>1.9036289092995512E-12</v>
       </c>
       <c r="S84" s="23">
-        <v>1.1124407655959028E-13</v>
+        <v>2.451769638850862E-14</v>
       </c>
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.3">
@@ -5297,7 +5285,7 @@
         <v>2</v>
       </c>
       <c r="C85">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D85">
         <v>5</v>
@@ -5309,34 +5297,34 @@
         <v>5</v>
       </c>
       <c r="G85">
-        <v>576</v>
+        <v>448</v>
       </c>
       <c r="H85" s="8">
-        <v>1.6319444444444445E-2</v>
+        <v>1.9642857142857146E-2</v>
       </c>
       <c r="I85" s="10">
-        <v>43.930902777777774</v>
+        <v>42.666964285714279</v>
       </c>
       <c r="J85" s="16">
-        <v>2.9625200000000002E-3</v>
+        <v>2.43888E-3</v>
       </c>
       <c r="K85" s="16">
-        <v>3.0337073399999999</v>
+        <v>2.1699046600000003</v>
       </c>
       <c r="L85" s="21">
-        <v>8.7563421659102526E-15</v>
+        <v>8.0746483171160317E-15</v>
       </c>
       <c r="M85" s="21">
-        <v>1.8086193569675066E-16</v>
+        <v>1.8361153524691382E-16</v>
       </c>
       <c r="Q85" s="16">
-        <v>2.6988541599999998</v>
+        <v>1.41559104</v>
       </c>
       <c r="R85" s="23">
-        <v>3.1965184679858536E-10</v>
+        <v>7.8049497441862349E-11</v>
       </c>
       <c r="S85" s="23">
-        <v>1.8248833852568277E-13</v>
+        <v>1.1124407655959028E-13</v>
       </c>
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.3">
@@ -5347,7 +5335,7 @@
         <v>2</v>
       </c>
       <c r="C86">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D86">
         <v>5</v>
@@ -5359,34 +5347,34 @@
         <v>5</v>
       </c>
       <c r="G86">
-        <v>720</v>
+        <v>576</v>
       </c>
       <c r="H86" s="8">
-        <v>1.7499999999999998E-2</v>
+        <v>1.6319444444444445E-2</v>
       </c>
       <c r="I86" s="10">
-        <v>45.905277777777783</v>
+        <v>43.930902777777774</v>
       </c>
       <c r="J86" s="16">
-        <v>3.6048000000000005E-3</v>
+        <v>2.9625200000000002E-3</v>
       </c>
       <c r="K86" s="16">
-        <v>4.1214200400000003</v>
+        <v>3.0337073399999999</v>
       </c>
       <c r="L86" s="21">
-        <v>8.1221604086442086E-15</v>
+        <v>8.7563421659102526E-15</v>
       </c>
       <c r="M86" s="21">
-        <v>1.7674696975267334E-16</v>
+        <v>1.8086193569675066E-16</v>
       </c>
       <c r="Q86" s="16">
-        <v>5.3663346399999998</v>
+        <v>2.6988541599999998</v>
       </c>
       <c r="R86" s="23">
-        <v>8.9366837878838275E-11</v>
+        <v>3.1965184679858536E-10</v>
       </c>
       <c r="S86" s="23">
-        <v>5.983322273343556E-13</v>
+        <v>1.8248833852568277E-13</v>
       </c>
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.3">
@@ -5397,7 +5385,7 @@
         <v>2</v>
       </c>
       <c r="C87">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D87">
         <v>5</v>
@@ -5409,34 +5397,34 @@
         <v>5</v>
       </c>
       <c r="G87">
-        <v>880</v>
+        <v>720</v>
       </c>
       <c r="H87" s="8">
-        <v>1.0909090909090908E-2</v>
+        <v>1.7499999999999998E-2</v>
       </c>
       <c r="I87" s="10">
-        <v>46.384545454545453</v>
+        <v>45.905277777777783</v>
       </c>
       <c r="J87" s="16">
-        <v>4.5217199999999999E-3</v>
+        <v>3.6048000000000005E-3</v>
       </c>
       <c r="K87" s="16">
-        <v>5.1804248600000005</v>
+        <v>4.1214200400000003</v>
       </c>
       <c r="L87" s="21">
-        <v>4.0563133109035229E-13</v>
+        <v>8.1221604086442086E-15</v>
       </c>
       <c r="M87" s="21">
-        <v>1.7946917554982332E-16</v>
+        <v>1.7674696975267334E-16</v>
       </c>
       <c r="Q87" s="16">
-        <v>8.6941763399999985</v>
+        <v>5.3663346399999998</v>
       </c>
       <c r="R87" s="23">
-        <v>3.4883819294068199E-10</v>
+        <v>8.9366837878838275E-11</v>
       </c>
       <c r="S87" s="23">
-        <v>1.266692535217473E-12</v>
+        <v>5.983322273343556E-13</v>
       </c>
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.3">
@@ -5447,7 +5435,7 @@
         <v>2</v>
       </c>
       <c r="C88">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D88">
         <v>5</v>
@@ -5456,37 +5444,37 @@
         <v>0</v>
       </c>
       <c r="F88">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G88">
-        <v>1056</v>
+        <v>880</v>
       </c>
       <c r="H88" s="8">
-        <v>1.3636363636363637E-2</v>
+        <v>1.0909090909090908E-2</v>
       </c>
       <c r="I88" s="10">
-        <v>47.596780303030307</v>
+        <v>46.384545454545453</v>
       </c>
       <c r="J88" s="16">
-        <v>5.1335600000000006E-3</v>
+        <v>4.5217199999999999E-3</v>
       </c>
       <c r="K88" s="16">
-        <v>6.70655512</v>
+        <v>5.1804248600000005</v>
       </c>
       <c r="L88" s="21">
-        <v>8.856099390063399E-15</v>
+        <v>4.0563133109035229E-13</v>
       </c>
       <c r="M88" s="21">
-        <v>1.8085618481595117E-16</v>
+        <v>1.7946917554982332E-16</v>
       </c>
       <c r="Q88" s="16">
-        <v>15.056374466666668</v>
+        <v>8.6941763399999985</v>
       </c>
       <c r="R88" s="23">
-        <v>2.4295018337047839E-8</v>
+        <v>3.4883819294068199E-10</v>
       </c>
       <c r="S88" s="23">
-        <v>2.308890906404235E-12</v>
+        <v>1.266692535217473E-12</v>
       </c>
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.3">
@@ -5497,7 +5485,7 @@
         <v>2</v>
       </c>
       <c r="C89">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D89">
         <v>5</v>
@@ -5509,34 +5497,34 @@
         <v>3</v>
       </c>
       <c r="G89">
-        <v>1248</v>
+        <v>1056</v>
       </c>
       <c r="H89" s="8">
-        <v>9.935897435897437E-3</v>
+        <v>1.3636363636363637E-2</v>
       </c>
       <c r="I89" s="10">
-        <v>48.495993589743591</v>
+        <v>47.596780303030307</v>
       </c>
       <c r="J89" s="16">
-        <v>6.1504000000000003E-3</v>
+        <v>5.1335600000000006E-3</v>
       </c>
       <c r="K89" s="16">
-        <v>8.1608353799999982</v>
+        <v>6.70655512</v>
       </c>
       <c r="L89" s="21">
-        <v>4.5313439140602873E-14</v>
+        <v>8.856099390063399E-15</v>
       </c>
       <c r="M89" s="21">
-        <v>1.7779168818308106E-16</v>
+        <v>1.8085618481595117E-16</v>
       </c>
       <c r="Q89" s="16">
-        <v>25.834941299999997</v>
+        <v>15.056374466666668</v>
       </c>
       <c r="R89" s="23">
-        <v>1.1219879282896385E-7</v>
+        <v>2.4295018337047839E-8</v>
       </c>
       <c r="S89" s="23">
-        <v>6.0061331322282475E-11</v>
+        <v>2.308890906404235E-12</v>
       </c>
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.3">
@@ -5547,46 +5535,46 @@
         <v>2</v>
       </c>
       <c r="C90">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D90">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E90">
         <v>0</v>
       </c>
       <c r="F90">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G90">
-        <v>1456</v>
+        <v>1248</v>
       </c>
       <c r="H90" s="8">
-        <v>1.510989010989011E-2</v>
+        <v>9.935897435897437E-3</v>
       </c>
       <c r="I90" s="10">
-        <v>50.130494505494504</v>
+        <v>48.495993589743591</v>
       </c>
       <c r="J90" s="16">
-        <v>7.1642999999999993E-3</v>
+        <v>6.1504000000000003E-3</v>
       </c>
       <c r="K90" s="16">
-        <v>10.554905466666666</v>
+        <v>8.1608353799999982</v>
       </c>
       <c r="L90" s="21">
-        <v>7.1176206096708818E-13</v>
+        <v>4.5313439140602873E-14</v>
       </c>
       <c r="M90" s="21">
-        <v>1.7861793287256898E-16</v>
+        <v>1.7779168818308106E-16</v>
       </c>
       <c r="Q90" s="16">
-        <v>43.764413300000001</v>
+        <v>25.834941299999997</v>
       </c>
       <c r="R90" s="23">
-        <v>4.2691807837727752E-8</v>
+        <v>1.1219879282896385E-7</v>
       </c>
       <c r="S90" s="23">
-        <v>6.2430990554405218E-11</v>
+        <v>6.0061331322282475E-11</v>
       </c>
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.3">
@@ -5597,7 +5585,7 @@
         <v>2</v>
       </c>
       <c r="C91">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D91">
         <v>3</v>
@@ -5609,34 +5597,34 @@
         <v>1</v>
       </c>
       <c r="G91">
-        <v>1680</v>
+        <v>1456</v>
       </c>
       <c r="H91" s="8">
-        <v>1.1309523809523809E-2</v>
+        <v>1.510989010989011E-2</v>
       </c>
       <c r="I91" s="10">
-        <v>50.704563492063492</v>
+        <v>50.130494505494504</v>
       </c>
       <c r="J91" s="16">
-        <v>8.1736666666666676E-3</v>
+        <v>7.1642999999999993E-3</v>
       </c>
       <c r="K91" s="16">
-        <v>12.699480933333334</v>
+        <v>10.554905466666666</v>
       </c>
       <c r="L91" s="21">
-        <v>8.8981459305272474E-15</v>
+        <v>7.1176206096708818E-13</v>
       </c>
       <c r="M91" s="21">
-        <v>1.7513656631602058E-16</v>
+        <v>1.7861793287256898E-16</v>
       </c>
       <c r="Q91" s="16">
-        <v>68.735169999999997</v>
+        <v>43.764413300000001</v>
       </c>
       <c r="R91" s="23">
-        <v>2.9854311789293022E-7</v>
+        <v>4.2691807837727752E-8</v>
       </c>
       <c r="S91" s="23">
-        <v>2.3696610952665727E-10</v>
+        <v>6.2430990554405218E-11</v>
       </c>
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.3">
@@ -5647,7 +5635,7 @@
         <v>2</v>
       </c>
       <c r="C92">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D92">
         <v>3</v>
@@ -5659,34 +5647,34 @@
         <v>1</v>
       </c>
       <c r="G92">
-        <v>1920</v>
+        <v>1680</v>
       </c>
       <c r="H92" s="8">
-        <v>1.2847222222222223E-2</v>
+        <v>1.1309523809523809E-2</v>
       </c>
       <c r="I92" s="10">
-        <v>51.958506944444444</v>
+        <v>50.704563492063492</v>
       </c>
       <c r="J92" s="16">
-        <v>9.1122333333333323E-3</v>
+        <v>8.1736666666666676E-3</v>
       </c>
       <c r="K92" s="16">
-        <v>15.405627433333331</v>
+        <v>12.699480933333334</v>
       </c>
       <c r="L92" s="21">
-        <v>8.5753805662679717E-15</v>
+        <v>8.8981459305272474E-15</v>
       </c>
       <c r="M92" s="21">
-        <v>1.7745128677302042E-16</v>
+        <v>1.7513656631602058E-16</v>
       </c>
       <c r="Q92" s="16">
-        <v>115.3274906</v>
+        <v>68.735169999999997</v>
       </c>
       <c r="R92" s="23">
-        <v>9.7650735782652114E-8</v>
+        <v>2.9854311789293022E-7</v>
       </c>
       <c r="S92" s="23">
-        <v>1.468131376872587E-10</v>
+        <v>2.3696610952665727E-10</v>
       </c>
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.3">
@@ -5694,49 +5682,49 @@
         <v>4</v>
       </c>
       <c r="B93">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C93">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D93">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E93">
         <v>0</v>
       </c>
       <c r="F93">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G93">
-        <v>256</v>
+        <v>1920</v>
       </c>
       <c r="H93" s="8">
-        <v>3.7499999999999999E-2</v>
+        <v>1.2847222222222223E-2</v>
       </c>
       <c r="I93" s="10">
-        <v>34.6796875</v>
+        <v>51.958506944444444</v>
       </c>
       <c r="J93" s="16">
-        <v>1.0819E-3</v>
+        <v>9.1122333333333323E-3</v>
       </c>
       <c r="K93" s="16">
-        <v>1.2695744000000002</v>
+        <v>15.405627433333331</v>
       </c>
       <c r="L93" s="21">
-        <v>2.0132970511526198E-14</v>
+        <v>8.5753805662679717E-15</v>
       </c>
       <c r="M93" s="21">
-        <v>3.1160955247749329E-16</v>
+        <v>1.7745128677302042E-16</v>
       </c>
       <c r="Q93" s="16">
-        <v>0.54818089999999997</v>
+        <v>115.3274906</v>
       </c>
       <c r="R93" s="23">
-        <v>4.6418020215540686E-13</v>
+        <v>9.7650735782652114E-8</v>
       </c>
       <c r="S93" s="23">
-        <v>4.7421697260468803E-15</v>
+        <v>1.468131376872587E-10</v>
       </c>
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.3">
@@ -5747,7 +5735,7 @@
         <v>3</v>
       </c>
       <c r="C94">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D94">
         <v>5</v>
@@ -5759,34 +5747,34 @@
         <v>5</v>
       </c>
       <c r="G94">
-        <v>640</v>
+        <v>256</v>
       </c>
       <c r="H94" s="8">
-        <v>4.4687500000000005E-2</v>
+        <v>3.7499999999999999E-2</v>
       </c>
       <c r="I94" s="10">
-        <v>37.266875000000006</v>
+        <v>34.6796875</v>
       </c>
       <c r="J94" s="16">
-        <v>1.9033400000000003E-3</v>
+        <v>1.0819E-3</v>
       </c>
       <c r="K94" s="16">
-        <v>3.4576043599999999</v>
+        <v>1.2695744000000002</v>
       </c>
       <c r="L94" s="21">
-        <v>1.7151996279412218E-14</v>
+        <v>2.0132970511526198E-14</v>
       </c>
       <c r="M94" s="21">
-        <v>2.7287804132474252E-16</v>
+        <v>3.1160955247749329E-16</v>
       </c>
       <c r="Q94" s="16">
-        <v>2.5991152799999995</v>
+        <v>0.54818089999999997</v>
       </c>
       <c r="R94" s="23">
-        <v>5.8968561566010554E-12</v>
+        <v>4.6418020215540686E-13</v>
       </c>
       <c r="S94" s="23">
-        <v>5.5666729068412767E-15</v>
+        <v>4.7421697260468803E-15</v>
       </c>
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.3">
@@ -5797,7 +5785,7 @@
         <v>3</v>
       </c>
       <c r="C95">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D95">
         <v>5</v>
@@ -5806,37 +5794,37 @@
         <v>0</v>
       </c>
       <c r="F95">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G95">
-        <v>1280</v>
+        <v>640</v>
       </c>
       <c r="H95" s="8">
-        <v>4.8437500000000001E-2</v>
+        <v>4.4687500000000005E-2</v>
       </c>
       <c r="I95" s="10">
-        <v>39.59796875</v>
+        <v>37.266875000000006</v>
       </c>
       <c r="J95" s="16">
-        <v>3.72822E-3</v>
+        <v>1.9033400000000003E-3</v>
       </c>
       <c r="K95" s="16">
-        <v>7.8842147200000001</v>
+        <v>3.4576043599999999</v>
       </c>
       <c r="L95" s="21">
-        <v>2.9964443174956343E-14</v>
+        <v>1.7151996279412218E-14</v>
       </c>
       <c r="M95" s="21">
-        <v>2.5838472390410206E-16</v>
+        <v>2.7287804132474252E-16</v>
       </c>
       <c r="Q95" s="16">
-        <v>13.694324433333334</v>
+        <v>2.5991152799999995</v>
       </c>
       <c r="R95" s="23">
-        <v>5.6072664396495966E-12</v>
+        <v>5.8968561566010554E-12</v>
       </c>
       <c r="S95" s="23">
-        <v>1.0970575168905956E-14</v>
+        <v>5.5666729068412767E-15</v>
       </c>
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.3">
@@ -5847,46 +5835,46 @@
         <v>3</v>
       </c>
       <c r="C96">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D96">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E96">
         <v>0</v>
       </c>
       <c r="F96">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G96">
-        <v>2240</v>
+        <v>1280</v>
       </c>
       <c r="H96" s="8">
-        <v>3.4375000000000003E-2</v>
+        <v>4.8437500000000001E-2</v>
       </c>
       <c r="I96" s="10">
-        <v>39.656845238095237</v>
+        <v>39.59796875</v>
       </c>
       <c r="J96" s="16">
-        <v>6.4512333333333338E-3</v>
+        <v>3.72822E-3</v>
       </c>
       <c r="K96" s="16">
-        <v>14.612070233333334</v>
+        <v>7.8842147200000001</v>
       </c>
       <c r="L96" s="21">
-        <v>1.0285622689536414E-12</v>
+        <v>2.9964443174956343E-14</v>
       </c>
       <c r="M96" s="21">
-        <v>2.4789962864686991E-16</v>
+        <v>2.5838472390410206E-16</v>
       </c>
       <c r="Q96" s="16">
-        <v>78.473416999999998</v>
+        <v>13.694324433333334</v>
       </c>
       <c r="R96" s="23">
-        <v>1.8499076792100177E-11</v>
+        <v>5.6072664396495966E-12</v>
       </c>
       <c r="S96" s="23">
-        <v>3.3888450136734267E-14</v>
+        <v>1.0970575168905956E-14</v>
       </c>
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.3">
@@ -5894,10 +5882,10 @@
         <v>4</v>
       </c>
       <c r="B97">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C97">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D97">
         <v>3</v>
@@ -5906,37 +5894,37 @@
         <v>0</v>
       </c>
       <c r="F97">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G97">
-        <v>1280</v>
+        <v>2240</v>
       </c>
       <c r="H97" s="8">
-        <v>7.239583333333334E-2</v>
+        <v>3.4375000000000003E-2</v>
       </c>
       <c r="I97" s="10">
-        <v>37.006510416666664</v>
+        <v>39.656845238095237</v>
       </c>
       <c r="J97" s="16">
-        <v>2.7899666666666664E-3</v>
+        <v>6.4512333333333338E-3</v>
       </c>
       <c r="K97" s="16">
-        <v>10.7165324</v>
+        <v>14.612070233333334</v>
       </c>
       <c r="L97" s="21">
-        <v>4.4504646015332152E-14</v>
+        <v>1.0285622689536414E-12</v>
       </c>
       <c r="M97" s="21">
-        <v>3.8130984615729509E-16</v>
+        <v>2.4789962864686991E-16</v>
       </c>
       <c r="Q97" s="16">
-        <v>26.523647033333333</v>
+        <v>78.473416999999998</v>
       </c>
       <c r="R97" s="23">
-        <v>4.1193002835668419E-11</v>
+        <v>1.8499076792100177E-11</v>
       </c>
       <c r="S97" s="23">
-        <v>8.1716021343870607E-15</v>
+        <v>3.3888450136734267E-14</v>
       </c>
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.3">
@@ -5947,87 +5935,87 @@
         <v>4</v>
       </c>
       <c r="C98">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D98">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E98">
         <v>0</v>
       </c>
       <c r="F98">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G98">
-        <v>3840</v>
+        <v>1280</v>
       </c>
       <c r="H98" s="8">
-        <v>6.458333333333334E-2</v>
+        <v>7.239583333333334E-2</v>
       </c>
       <c r="I98" s="10">
-        <v>38.025260416666669</v>
+        <v>37.006510416666664</v>
       </c>
       <c r="J98" s="16">
-        <v>7.5215000000000004E-3</v>
+        <v>2.7899666666666664E-3</v>
       </c>
       <c r="K98" s="16">
-        <v>33.928097700000002</v>
+        <v>10.7165324</v>
       </c>
       <c r="L98" s="21">
-        <v>2.8704818616543717E-14</v>
+        <v>4.4504646015332152E-14</v>
       </c>
       <c r="M98" s="21">
-        <v>3.4110084723815503E-16</v>
+        <v>3.8130984615729509E-16</v>
+      </c>
+      <c r="Q98" s="16">
+        <v>26.523647033333333</v>
+      </c>
+      <c r="R98" s="23">
+        <v>4.1193002835668419E-11</v>
+      </c>
+      <c r="S98" s="23">
+        <v>8.1716021343870607E-15</v>
       </c>
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A99">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B99">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C99">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D99">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E99">
         <v>0</v>
       </c>
       <c r="F99">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G99">
-        <v>75</v>
+        <v>3840</v>
       </c>
       <c r="H99" s="8">
-        <v>3.2000000000000001E-2</v>
+        <v>6.458333333333334E-2</v>
       </c>
       <c r="I99" s="10">
-        <v>34.058666666666667</v>
+        <v>38.025260416666669</v>
       </c>
       <c r="J99" s="16">
-        <v>6.623E-4</v>
+        <v>7.5215000000000004E-3</v>
       </c>
       <c r="K99" s="16">
-        <v>0.31772778000000002</v>
+        <v>33.928097700000002</v>
       </c>
       <c r="L99" s="21">
-        <v>8.1802588652744995E-15</v>
+        <v>2.8704818616543717E-14</v>
       </c>
       <c r="M99" s="21">
-        <v>2.7054990438010407E-16</v>
-      </c>
-      <c r="Q99" s="16">
-        <v>9.5071459999999997E-2</v>
-      </c>
-      <c r="R99" s="23">
-        <v>2.1230176129388547E-13</v>
-      </c>
-      <c r="S99" s="23">
-        <v>2.6554082342794527E-15</v>
+        <v>3.4110084723815503E-16</v>
       </c>
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.3">
@@ -6038,7 +6026,7 @@
         <v>2</v>
       </c>
       <c r="C100">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D100">
         <v>5</v>
@@ -6050,34 +6038,34 @@
         <v>5</v>
       </c>
       <c r="G100">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="H100" s="8">
-        <v>3.7333333333333329E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="I100" s="10">
-        <v>36.805333333333337</v>
+        <v>34.058666666666667</v>
       </c>
       <c r="J100" s="16">
-        <v>8.6505999999999996E-4</v>
+        <v>6.623E-4</v>
       </c>
       <c r="K100" s="16">
-        <v>0.68472791999999993</v>
+        <v>0.31772778000000002</v>
       </c>
       <c r="L100" s="21">
-        <v>7.9992386291296098E-14</v>
+        <v>8.1802588652744995E-15</v>
       </c>
       <c r="M100" s="21">
-        <v>2.3437174106603008E-16</v>
+        <v>2.7054990438010407E-16</v>
       </c>
       <c r="Q100" s="16">
-        <v>0.20571149999999999</v>
+        <v>9.5071459999999997E-2</v>
       </c>
       <c r="R100" s="23">
-        <v>3.9276827367189106E-13</v>
+        <v>2.1230176129388547E-13</v>
       </c>
       <c r="S100" s="23">
-        <v>3.887301769157956E-15</v>
+        <v>2.6554082342794527E-15</v>
       </c>
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.3">
@@ -6088,7 +6076,7 @@
         <v>2</v>
       </c>
       <c r="C101">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D101">
         <v>5</v>
@@ -6100,34 +6088,34 @@
         <v>5</v>
       </c>
       <c r="G101">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="H101" s="8">
-        <v>2.7199999999999998E-2</v>
+        <v>3.7333333333333329E-2</v>
       </c>
       <c r="I101" s="10">
-        <v>37.944000000000003</v>
+        <v>36.805333333333337</v>
       </c>
       <c r="J101" s="16">
-        <v>1.1263600000000001E-3</v>
+        <v>8.6505999999999996E-4</v>
       </c>
       <c r="K101" s="16">
-        <v>1.1483679399999998</v>
+        <v>0.68472791999999993</v>
       </c>
       <c r="L101" s="21">
-        <v>1.4703385801104632E-14</v>
+        <v>7.9992386291296098E-14</v>
       </c>
       <c r="M101" s="21">
-        <v>2.249163067383749E-16</v>
+        <v>2.3437174106603008E-16</v>
       </c>
       <c r="Q101" s="16">
-        <v>0.45794532000000004</v>
+        <v>0.20571149999999999</v>
       </c>
       <c r="R101" s="23">
-        <v>7.9015136443126549E-13</v>
+        <v>3.9276827367189106E-13</v>
       </c>
       <c r="S101" s="23">
-        <v>1.0980834697690558E-14</v>
+        <v>3.887301769157956E-15</v>
       </c>
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.3">
@@ -6138,7 +6126,7 @@
         <v>2</v>
       </c>
       <c r="C102">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D102">
         <v>5</v>
@@ -6150,34 +6138,34 @@
         <v>5</v>
       </c>
       <c r="G102">
-        <v>375</v>
+        <v>250</v>
       </c>
       <c r="H102" s="8">
-        <v>2.4E-2</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="I102" s="10">
-        <v>39.789333333333332</v>
+        <v>37.944000000000003</v>
       </c>
       <c r="J102" s="16">
-        <v>1.5102200000000001E-3</v>
+        <v>1.1263600000000001E-3</v>
       </c>
       <c r="K102" s="16">
-        <v>1.8615628799999999</v>
+        <v>1.1483679399999998</v>
       </c>
       <c r="L102" s="21">
-        <v>1.5468578750210955E-14</v>
+        <v>1.4703385801104632E-14</v>
       </c>
       <c r="M102" s="21">
-        <v>2.2084568777386575E-16</v>
+        <v>2.249163067383749E-16</v>
       </c>
       <c r="Q102" s="16">
-        <v>0.94974728000000008</v>
+        <v>0.45794532000000004</v>
       </c>
       <c r="R102" s="23">
-        <v>2.9094147727193586E-12</v>
+        <v>7.9015136443126549E-13</v>
       </c>
       <c r="S102" s="23">
-        <v>7.9947913515779821E-14</v>
+        <v>1.0980834697690558E-14</v>
       </c>
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.3">
@@ -6188,7 +6176,7 @@
         <v>2</v>
       </c>
       <c r="C103">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D103">
         <v>5</v>
@@ -6200,34 +6188,34 @@
         <v>5</v>
       </c>
       <c r="G103">
-        <v>525</v>
+        <v>375</v>
       </c>
       <c r="H103" s="8">
-        <v>2.1333333333333333E-2</v>
+        <v>2.4E-2</v>
       </c>
       <c r="I103" s="10">
-        <v>41.500571428571426</v>
+        <v>39.789333333333332</v>
       </c>
       <c r="J103" s="16">
-        <v>1.9948000000000001E-3</v>
+        <v>1.5102200000000001E-3</v>
       </c>
       <c r="K103" s="16">
-        <v>2.8250143000000003</v>
+        <v>1.8615628799999999</v>
       </c>
       <c r="L103" s="21">
-        <v>1.4833348118405114E-14</v>
+        <v>1.5468578750210955E-14</v>
       </c>
       <c r="M103" s="21">
-        <v>2.1174835996058322E-16</v>
+        <v>2.2084568777386575E-16</v>
       </c>
       <c r="Q103" s="16">
-        <v>2.0045685999999998</v>
+        <v>0.94974728000000008</v>
       </c>
       <c r="R103" s="23">
-        <v>9.6685578236614547E-12</v>
+        <v>2.9094147727193586E-12</v>
       </c>
       <c r="S103" s="23">
-        <v>5.0820155852136305E-14</v>
+        <v>7.9947913515779821E-14</v>
       </c>
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.3">
@@ -6238,7 +6226,7 @@
         <v>2</v>
       </c>
       <c r="C104">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D104">
         <v>5</v>
@@ -6250,34 +6238,34 @@
         <v>5</v>
       </c>
       <c r="G104">
-        <v>700</v>
+        <v>525</v>
       </c>
       <c r="H104" s="8">
-        <v>2.4285714285714285E-2</v>
+        <v>2.1333333333333333E-2</v>
       </c>
       <c r="I104" s="10">
-        <v>43.141428571428577</v>
+        <v>41.500571428571426</v>
       </c>
       <c r="J104" s="16">
-        <v>2.5738999999999996E-3</v>
+        <v>1.9948000000000001E-3</v>
       </c>
       <c r="K104" s="16">
-        <v>4.0745186200000001</v>
+        <v>2.8250143000000003</v>
       </c>
       <c r="L104" s="21">
-        <v>3.8779438915317176E-13</v>
+        <v>1.4833348118405114E-14</v>
       </c>
       <c r="M104" s="21">
-        <v>2.1531211961687913E-16</v>
+        <v>2.1174835996058322E-16</v>
       </c>
       <c r="Q104" s="16">
-        <v>4.3959003600000006</v>
+        <v>2.0045685999999998</v>
       </c>
       <c r="R104" s="23">
-        <v>1.5402273032896525E-10</v>
+        <v>9.6685578236614547E-12</v>
       </c>
       <c r="S104" s="23">
-        <v>1.3596143244377566E-13</v>
+        <v>5.0820155852136305E-14</v>
       </c>
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.3">
@@ -6288,7 +6276,7 @@
         <v>2</v>
       </c>
       <c r="C105">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D105">
         <v>5</v>
@@ -6300,34 +6288,34 @@
         <v>5</v>
       </c>
       <c r="G105">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="H105" s="8">
-        <v>2.0222222222222221E-2</v>
+        <v>2.4285714285714285E-2</v>
       </c>
       <c r="I105" s="10">
-        <v>44.225555555555552</v>
+        <v>43.141428571428577</v>
       </c>
       <c r="J105" s="16">
-        <v>2.9292000000000003E-3</v>
+        <v>2.5738999999999996E-3</v>
       </c>
       <c r="K105" s="16">
-        <v>5.5390185399999998</v>
+        <v>4.0745186200000001</v>
       </c>
       <c r="L105" s="21">
-        <v>1.4901997469166348E-14</v>
+        <v>3.8779438915317176E-13</v>
       </c>
       <c r="M105" s="21">
-        <v>2.1025872780187197E-16</v>
+        <v>2.1531211961687913E-16</v>
       </c>
       <c r="Q105" s="16">
-        <v>8.3908084400000007</v>
+        <v>4.3959003600000006</v>
       </c>
       <c r="R105" s="23">
-        <v>9.3880357060867293E-11</v>
+        <v>1.5402273032896525E-10</v>
       </c>
       <c r="S105" s="23">
-        <v>3.3585867021730076E-13</v>
+        <v>1.3596143244377566E-13</v>
       </c>
     </row>
     <row r="106" spans="1:19" x14ac:dyDescent="0.3">
@@ -6338,7 +6326,7 @@
         <v>2</v>
       </c>
       <c r="C106">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D106">
         <v>5</v>
@@ -6347,37 +6335,37 @@
         <v>0</v>
       </c>
       <c r="F106">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G106">
-        <v>1125</v>
+        <v>900</v>
       </c>
       <c r="H106" s="8">
-        <v>1.2977777777777777E-2</v>
+        <v>2.0222222222222221E-2</v>
       </c>
       <c r="I106" s="10">
-        <v>45.380622222222222</v>
+        <v>44.225555555555552</v>
       </c>
       <c r="J106" s="16">
-        <v>3.96716E-3</v>
+        <v>2.9292000000000003E-3</v>
       </c>
       <c r="K106" s="16">
-        <v>7.6967464799999998</v>
+        <v>5.5390185399999998</v>
       </c>
       <c r="L106" s="21">
-        <v>1.5187790760508941E-14</v>
+        <v>1.4901997469166348E-14</v>
       </c>
       <c r="M106" s="21">
-        <v>2.0590819941881997E-16</v>
+        <v>2.1025872780187197E-16</v>
       </c>
       <c r="Q106" s="16">
-        <v>16.5025662</v>
+        <v>8.3908084400000007</v>
       </c>
       <c r="R106" s="23">
-        <v>4.6948410934586531E-9</v>
+        <v>9.3880357060867293E-11</v>
       </c>
       <c r="S106" s="23">
-        <v>1.2651012022538633E-11</v>
+        <v>3.3585867021730076E-13</v>
       </c>
     </row>
     <row r="107" spans="1:19" x14ac:dyDescent="0.3">
@@ -6388,7 +6376,7 @@
         <v>2</v>
       </c>
       <c r="C107">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D107">
         <v>5</v>
@@ -6400,34 +6388,34 @@
         <v>3</v>
       </c>
       <c r="G107">
-        <v>1375</v>
+        <v>1125</v>
       </c>
       <c r="H107" s="8">
-        <v>1.5854545454545454E-2</v>
+        <v>1.2977777777777777E-2</v>
       </c>
       <c r="I107" s="10">
-        <v>46.487854545454546</v>
+        <v>45.380622222222222</v>
       </c>
       <c r="J107" s="16">
-        <v>4.53806E-3</v>
+        <v>3.96716E-3</v>
       </c>
       <c r="K107" s="16">
-        <v>9.8030528199999996</v>
+        <v>7.6967464799999998</v>
       </c>
       <c r="L107" s="21">
-        <v>4.6464405109889013E-14</v>
+        <v>1.5187790760508941E-14</v>
       </c>
       <c r="M107" s="21">
-        <v>2.068181647074715E-16</v>
+        <v>2.0590819941881997E-16</v>
       </c>
       <c r="Q107" s="16">
-        <v>31.790000933333335</v>
+        <v>16.5025662</v>
       </c>
       <c r="R107" s="23">
-        <v>4.1617999672704015E-9</v>
+        <v>4.6948410934586531E-9</v>
       </c>
       <c r="S107" s="23">
-        <v>1.6428829304690858E-12</v>
+        <v>1.2651012022538633E-11</v>
       </c>
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.3">
@@ -6435,10 +6423,10 @@
         <v>5</v>
       </c>
       <c r="B108">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C108">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D108">
         <v>5</v>
@@ -6447,37 +6435,37 @@
         <v>0</v>
       </c>
       <c r="F108">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G108">
-        <v>500</v>
+        <v>1375</v>
       </c>
       <c r="H108" s="8">
-        <v>6.5200000000000008E-2</v>
+        <v>1.5854545454545454E-2</v>
       </c>
       <c r="I108" s="10">
-        <v>35.793599999999998</v>
+        <v>46.487854545454546</v>
       </c>
       <c r="J108" s="16">
-        <v>1.0643599999999999E-3</v>
+        <v>4.53806E-3</v>
       </c>
       <c r="K108" s="16">
-        <v>3.2660372600000001</v>
+        <v>9.8030528199999996</v>
       </c>
       <c r="L108" s="21">
-        <v>4.150742209884161E-14</v>
+        <v>4.6464405109889013E-14</v>
       </c>
       <c r="M108" s="21">
-        <v>3.7494034505499536E-16</v>
+        <v>2.068181647074715E-16</v>
       </c>
       <c r="Q108" s="16">
-        <v>1.7813614600000001</v>
+        <v>31.790000933333335</v>
       </c>
       <c r="R108" s="23">
-        <v>3.6171699606032962E-13</v>
+        <v>4.1617999672704015E-9</v>
       </c>
       <c r="S108" s="23">
-        <v>5.1917279638947215E-15</v>
+        <v>1.6428829304690858E-12</v>
       </c>
     </row>
     <row r="109" spans="1:19" x14ac:dyDescent="0.3">
@@ -6488,7 +6476,7 @@
         <v>3</v>
       </c>
       <c r="C109">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D109">
         <v>5</v>
@@ -6500,34 +6488,34 @@
         <v>5</v>
       </c>
       <c r="G109">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="H109" s="8">
-        <v>4.9439999999999998E-2</v>
+        <v>6.5200000000000008E-2</v>
       </c>
       <c r="I109" s="10">
-        <v>36.797759999999997</v>
+        <v>35.793599999999998</v>
       </c>
       <c r="J109" s="16">
-        <v>2.25494E-3</v>
+        <v>1.0643599999999999E-3</v>
       </c>
       <c r="K109" s="16">
-        <v>8.1999447800000009</v>
+        <v>3.2660372600000001</v>
       </c>
       <c r="L109" s="21">
-        <v>3.6750446427367134E-14</v>
+        <v>4.150742209884161E-14</v>
       </c>
       <c r="M109" s="21">
-        <v>3.312044730280428E-16</v>
+        <v>3.7494034505499536E-16</v>
       </c>
       <c r="Q109" s="16">
-        <v>12.733139099999999</v>
+        <v>1.7813614600000001</v>
       </c>
       <c r="R109" s="23">
-        <v>5.3492872272192522E-12</v>
+        <v>3.6171699606032962E-13</v>
       </c>
       <c r="S109" s="23">
-        <v>4.4684299183482005E-14</v>
+        <v>5.1917279638947215E-15</v>
       </c>
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.3">
@@ -6538,46 +6526,46 @@
         <v>3</v>
       </c>
       <c r="C110">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D110">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E110">
         <v>0</v>
       </c>
       <c r="F110">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G110">
-        <v>2500</v>
+        <v>1250</v>
       </c>
       <c r="H110" s="8">
-        <v>4.2533333333333333E-2</v>
+        <v>4.9439999999999998E-2</v>
       </c>
       <c r="I110" s="10">
-        <v>38.0944</v>
+        <v>36.797759999999997</v>
       </c>
       <c r="J110" s="16">
-        <v>3.6237333333333337E-3</v>
+        <v>2.25494E-3</v>
       </c>
       <c r="K110" s="16">
-        <v>18.169718133333333</v>
+        <v>8.1999447800000009</v>
       </c>
       <c r="L110" s="21">
-        <v>3.5960977846467271E-14</v>
+        <v>3.6750446427367134E-14</v>
       </c>
       <c r="M110" s="21">
-        <v>3.1375495388067941E-16</v>
+        <v>3.312044730280428E-16</v>
       </c>
       <c r="Q110" s="16">
-        <v>106.53776413333333</v>
+        <v>12.733139099999999</v>
       </c>
       <c r="R110" s="23">
-        <v>3.5097177365450714E-11</v>
+        <v>5.3492872272192522E-12</v>
       </c>
       <c r="S110" s="23">
-        <v>3.9393172071118404E-14</v>
+        <v>4.4684299183482005E-14</v>
       </c>
     </row>
     <row r="111" spans="1:19" x14ac:dyDescent="0.3">
@@ -6588,37 +6576,46 @@
         <v>3</v>
       </c>
       <c r="C111">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D111">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E111">
         <v>0</v>
       </c>
       <c r="F111">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G111">
-        <v>4375</v>
+        <v>2500</v>
       </c>
       <c r="H111" s="8">
-        <v>4.3428571428571427E-2</v>
+        <v>4.2533333333333333E-2</v>
       </c>
       <c r="I111" s="10">
-        <v>40.537371428571426</v>
+        <v>38.0944</v>
       </c>
       <c r="J111" s="16">
-        <v>7.2175E-3</v>
+        <v>3.6237333333333337E-3</v>
       </c>
       <c r="K111" s="16">
-        <v>40.470895000000006</v>
+        <v>18.169718133333333</v>
       </c>
       <c r="L111" s="21">
-        <v>3.7320878384676091E-12</v>
+        <v>3.5960977846467271E-14</v>
       </c>
       <c r="M111" s="21">
-        <v>3.035776384633188E-16</v>
+        <v>3.1375495388067941E-16</v>
+      </c>
+      <c r="Q111" s="16">
+        <v>106.53776413333333</v>
+      </c>
+      <c r="R111" s="23">
+        <v>3.5097177365450714E-11</v>
+      </c>
+      <c r="S111" s="23">
+        <v>3.9393172071118404E-14</v>
       </c>
     </row>
     <row r="112" spans="1:19" x14ac:dyDescent="0.3">
@@ -6626,10 +6623,10 @@
         <v>5</v>
       </c>
       <c r="B112">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C112">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D112">
         <v>1</v>
@@ -6641,75 +6638,66 @@
         <v>0</v>
       </c>
       <c r="G112">
-        <v>3125</v>
+        <v>4375</v>
       </c>
       <c r="H112" s="8">
-        <v>9.1200000000000003E-2</v>
+        <v>4.3428571428571427E-2</v>
       </c>
       <c r="I112" s="10">
-        <v>36.86112</v>
+        <v>40.537371428571426</v>
       </c>
       <c r="J112" s="16">
-        <v>3.5699999999999998E-3</v>
+        <v>7.2175E-3</v>
       </c>
       <c r="K112" s="16">
-        <v>36.600457300000002</v>
+        <v>40.470895000000006</v>
       </c>
       <c r="L112" s="21">
-        <v>7.586296295965602E-14</v>
+        <v>3.7320878384676091E-12</v>
       </c>
       <c r="M112" s="21">
-        <v>5.0452484515548831E-16</v>
+        <v>3.035776384633188E-16</v>
       </c>
     </row>
     <row r="113" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A113">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B113">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C113">
         <v>2</v>
       </c>
       <c r="D113">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E113">
         <v>0</v>
       </c>
       <c r="F113">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G113">
-        <v>108</v>
+        <v>3125</v>
       </c>
       <c r="H113" s="8">
-        <v>3.7037037037037035E-2</v>
+        <v>9.1200000000000003E-2</v>
       </c>
       <c r="I113" s="10">
-        <v>34.296296296296291</v>
+        <v>36.86112</v>
       </c>
       <c r="J113" s="16">
-        <v>5.7476000000000001E-4</v>
+        <v>3.5699999999999998E-3</v>
       </c>
       <c r="K113" s="16">
-        <v>0.49949194000000008</v>
+        <v>36.600457300000002</v>
       </c>
       <c r="L113" s="21">
-        <v>3.2951693518883698E-14</v>
+        <v>7.586296295965602E-14</v>
       </c>
       <c r="M113" s="21">
-        <v>3.2604089195961668E-16</v>
-      </c>
-      <c r="Q113" s="16">
-        <v>0.15657246</v>
-      </c>
-      <c r="R113" s="23">
-        <v>6.5121299890427066E-13</v>
-      </c>
-      <c r="S113" s="23">
-        <v>5.8327545996067954E-15</v>
+        <v>5.0452484515548831E-16</v>
       </c>
     </row>
     <row r="114" spans="1:19" x14ac:dyDescent="0.3">
@@ -6720,7 +6708,7 @@
         <v>2</v>
       </c>
       <c r="C114">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D114">
         <v>5</v>
@@ -6732,34 +6720,34 @@
         <v>5</v>
       </c>
       <c r="G114">
-        <v>216</v>
+        <v>108</v>
       </c>
       <c r="H114" s="8">
-        <v>1.8518518518518517E-2</v>
+        <v>3.7037037037037035E-2</v>
       </c>
       <c r="I114" s="10">
-        <v>35.411111111111111</v>
+        <v>34.296296296296291</v>
       </c>
       <c r="J114" s="16">
-        <v>8.6555999999999992E-4</v>
+        <v>5.7476000000000001E-4</v>
       </c>
       <c r="K114" s="16">
-        <v>0.96189133999999998</v>
+        <v>0.49949194000000008</v>
       </c>
       <c r="L114" s="21">
-        <v>2.2280773584797067E-14</v>
+        <v>3.2951693518883698E-14</v>
       </c>
       <c r="M114" s="21">
-        <v>2.775353550537815E-16</v>
+        <v>3.2604089195961668E-16</v>
       </c>
       <c r="Q114" s="16">
-        <v>0.38666301999999997</v>
+        <v>0.15657246</v>
       </c>
       <c r="R114" s="23">
-        <v>1.4114124593626313E-13</v>
+        <v>6.5121299890427066E-13</v>
       </c>
       <c r="S114" s="23">
-        <v>5.8111683878486103E-15</v>
+        <v>5.8327545996067954E-15</v>
       </c>
     </row>
     <row r="115" spans="1:19" x14ac:dyDescent="0.3">
@@ -6770,7 +6758,7 @@
         <v>2</v>
       </c>
       <c r="C115">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D115">
         <v>5</v>
@@ -6782,34 +6770,34 @@
         <v>5</v>
       </c>
       <c r="G115">
-        <v>360</v>
+        <v>216</v>
       </c>
       <c r="H115" s="8">
-        <v>2.6111111111111113E-2</v>
+        <v>1.8518518518518517E-2</v>
       </c>
       <c r="I115" s="10">
-        <v>38.152222222222221</v>
+        <v>35.411111111111111</v>
       </c>
       <c r="J115" s="16">
-        <v>1.1808600000000002E-3</v>
+        <v>8.6555999999999992E-4</v>
       </c>
       <c r="K115" s="16">
-        <v>1.7728660199999999</v>
+        <v>0.96189133999999998</v>
       </c>
       <c r="L115" s="21">
-        <v>2.2335024315275464E-14</v>
+        <v>2.2280773584797067E-14</v>
       </c>
       <c r="M115" s="21">
-        <v>2.6826869574784005E-16</v>
+        <v>2.775353550537815E-16</v>
       </c>
       <c r="Q115" s="16">
-        <v>0.89140035999999989</v>
+        <v>0.38666301999999997</v>
       </c>
       <c r="R115" s="23">
-        <v>3.4187730159447699E-12</v>
+        <v>1.4114124593626313E-13</v>
       </c>
       <c r="S115" s="23">
-        <v>1.6614278870848769E-14</v>
+        <v>5.8111683878486103E-15</v>
       </c>
     </row>
     <row r="116" spans="1:19" x14ac:dyDescent="0.3">
@@ -6820,7 +6808,7 @@
         <v>2</v>
       </c>
       <c r="C116">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D116">
         <v>5</v>
@@ -6832,34 +6820,34 @@
         <v>5</v>
       </c>
       <c r="G116">
-        <v>540</v>
+        <v>360</v>
       </c>
       <c r="H116" s="8">
-        <v>1.740740740740741E-2</v>
+        <v>2.6111111111111113E-2</v>
       </c>
       <c r="I116" s="10">
-        <v>38.810740740740741</v>
+        <v>38.152222222222221</v>
       </c>
       <c r="J116" s="16">
-        <v>1.5954200000000002E-3</v>
+        <v>1.1808600000000002E-3</v>
       </c>
       <c r="K116" s="16">
-        <v>2.7022699399999999</v>
+        <v>1.7728660199999999</v>
       </c>
       <c r="L116" s="21">
-        <v>4.2929370064810047E-14</v>
+        <v>2.2335024315275464E-14</v>
       </c>
       <c r="M116" s="21">
-        <v>2.5682826709524424E-16</v>
+        <v>2.6826869574784005E-16</v>
       </c>
       <c r="Q116" s="16">
-        <v>2.0624484000000001</v>
+        <v>0.89140035999999989</v>
       </c>
       <c r="R116" s="23">
-        <v>2.8885148571738064E-12</v>
+        <v>3.4187730159447699E-12</v>
       </c>
       <c r="S116" s="23">
-        <v>3.3668543790314038E-14</v>
+        <v>1.6614278870848769E-14</v>
       </c>
     </row>
     <row r="117" spans="1:19" x14ac:dyDescent="0.3">
@@ -6870,7 +6858,7 @@
         <v>2</v>
       </c>
       <c r="C117">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D117">
         <v>5</v>
@@ -6882,34 +6870,34 @@
         <v>5</v>
       </c>
       <c r="G117">
-        <v>756</v>
+        <v>540</v>
       </c>
       <c r="H117" s="8">
-        <v>2.1693121693121691E-2</v>
+        <v>1.740740740740741E-2</v>
       </c>
       <c r="I117" s="10">
-        <v>41.141269841269839</v>
+        <v>38.810740740740741</v>
       </c>
       <c r="J117" s="16">
-        <v>2.0802400000000006E-3</v>
+        <v>1.5954200000000002E-3</v>
       </c>
       <c r="K117" s="16">
-        <v>4.4196238999999995</v>
+        <v>2.7022699399999999</v>
       </c>
       <c r="L117" s="21">
-        <v>2.4881551421311994E-14</v>
+        <v>4.2929370064810047E-14</v>
       </c>
       <c r="M117" s="21">
-        <v>2.5134843055559786E-16</v>
+        <v>2.5682826709524424E-16</v>
       </c>
       <c r="Q117" s="16">
-        <v>4.7410546200000008</v>
+        <v>2.0624484000000001</v>
       </c>
       <c r="R117" s="23">
-        <v>1.527669279158425E-11</v>
+        <v>2.8885148571738064E-12</v>
       </c>
       <c r="S117" s="23">
-        <v>5.4042023543274418E-14</v>
+        <v>3.3668543790314038E-14</v>
       </c>
     </row>
     <row r="118" spans="1:19" x14ac:dyDescent="0.3">
@@ -6920,7 +6908,7 @@
         <v>2</v>
       </c>
       <c r="C118">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D118">
         <v>5</v>
@@ -6929,37 +6917,37 @@
         <v>0</v>
       </c>
       <c r="F118">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G118">
-        <v>1008</v>
+        <v>756</v>
       </c>
       <c r="H118" s="8">
-        <v>2.103174603174603E-2</v>
+        <v>2.1693121693121691E-2</v>
       </c>
       <c r="I118" s="10">
-        <v>42.817261904761907</v>
+        <v>41.141269841269839</v>
       </c>
       <c r="J118" s="16">
-        <v>2.6401599999999999E-3</v>
+        <v>2.0802400000000006E-3</v>
       </c>
       <c r="K118" s="16">
-        <v>6.8269274400000004</v>
+        <v>4.4196238999999995</v>
       </c>
       <c r="L118" s="21">
-        <v>3.989523845769286E-13</v>
+        <v>2.4881551421311994E-14</v>
       </c>
       <c r="M118" s="21">
-        <v>2.4368210289639596E-16</v>
+        <v>2.5134843055559786E-16</v>
       </c>
       <c r="Q118" s="16">
-        <v>10.820841566666667</v>
+        <v>4.7410546200000008</v>
       </c>
       <c r="R118" s="23">
-        <v>5.4407729093785094E-10</v>
+        <v>1.527669279158425E-11</v>
       </c>
       <c r="S118" s="23">
-        <v>2.2454569809768172E-13</v>
+        <v>5.4042023543274418E-14</v>
       </c>
     </row>
     <row r="119" spans="1:19" x14ac:dyDescent="0.3">
@@ -6970,7 +6958,7 @@
         <v>2</v>
       </c>
       <c r="C119">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D119">
         <v>5</v>
@@ -6982,34 +6970,34 @@
         <v>3</v>
       </c>
       <c r="G119">
-        <v>1296</v>
+        <v>1008</v>
       </c>
       <c r="H119" s="8">
-        <v>1.1574074074074075E-2</v>
+        <v>2.103174603174603E-2</v>
       </c>
       <c r="I119" s="10">
-        <v>43.284104938271604</v>
+        <v>42.817261904761907</v>
       </c>
       <c r="J119" s="16">
-        <v>3.5624599999999999E-3</v>
+        <v>2.6401599999999999E-3</v>
       </c>
       <c r="K119" s="16">
-        <v>8.5879345600000008</v>
+        <v>6.8269274400000004</v>
       </c>
       <c r="L119" s="21">
-        <v>2.8940116364988023E-14</v>
+        <v>3.989523845769286E-13</v>
       </c>
       <c r="M119" s="21">
-        <v>2.38730216706383E-16</v>
+        <v>2.4368210289639596E-16</v>
       </c>
       <c r="Q119" s="16">
-        <v>23.0620048</v>
+        <v>10.820841566666667</v>
       </c>
       <c r="R119" s="23">
-        <v>1.6392681843978063E-9</v>
+        <v>5.4407729093785094E-10</v>
       </c>
       <c r="S119" s="23">
-        <v>3.8379790369403259E-12</v>
+        <v>2.2454569809768172E-13</v>
       </c>
     </row>
     <row r="120" spans="1:19" x14ac:dyDescent="0.3">
@@ -7020,46 +7008,46 @@
         <v>2</v>
       </c>
       <c r="C120">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D120">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E120">
         <v>0</v>
       </c>
       <c r="F120">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G120">
-        <v>1620</v>
+        <v>1296</v>
       </c>
       <c r="H120" s="8">
-        <v>1.5637860082304524E-2</v>
+        <v>1.1574074074074075E-2</v>
       </c>
       <c r="I120" s="10">
-        <v>45.101851851851855</v>
+        <v>43.284104938271604</v>
       </c>
       <c r="J120" s="16">
-        <v>5.1473333333333336E-3</v>
+        <v>3.5624599999999999E-3</v>
       </c>
       <c r="K120" s="16">
-        <v>11.7958102</v>
+        <v>8.5879345600000008</v>
       </c>
       <c r="L120" s="21">
-        <v>2.7295618335376128E-14</v>
+        <v>2.8940116364988023E-14</v>
       </c>
       <c r="M120" s="21">
-        <v>2.338866286165698E-16</v>
+        <v>2.38730216706383E-16</v>
       </c>
       <c r="Q120" s="16">
-        <v>46.985986799999999</v>
+        <v>23.0620048</v>
       </c>
       <c r="R120" s="23">
-        <v>1.0093041449742465E-9</v>
+        <v>1.6392681843978063E-9</v>
       </c>
       <c r="S120" s="23">
-        <v>7.5560159000718528E-13</v>
+        <v>3.8379790369403259E-12</v>
       </c>
     </row>
     <row r="121" spans="1:19" x14ac:dyDescent="0.3">
@@ -7070,7 +7058,7 @@
         <v>2</v>
       </c>
       <c r="C121">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D121">
         <v>3</v>
@@ -7082,34 +7070,34 @@
         <v>1</v>
       </c>
       <c r="G121">
-        <v>1980</v>
+        <v>1620</v>
       </c>
       <c r="H121" s="8">
-        <v>1.8013468013468013E-2</v>
+        <v>1.5637860082304524E-2</v>
       </c>
       <c r="I121" s="10">
-        <v>46.935690235690238</v>
+        <v>45.101851851851855</v>
       </c>
       <c r="J121" s="16">
-        <v>6.3254666666666673E-3</v>
+        <v>5.1473333333333336E-3</v>
       </c>
       <c r="K121" s="16">
-        <v>16.711406533333331</v>
+        <v>11.7958102</v>
       </c>
       <c r="L121" s="21">
-        <v>2.6698552285433069E-14</v>
+        <v>2.7295618335376128E-14</v>
       </c>
       <c r="M121" s="21">
-        <v>2.378899902841658E-16</v>
+        <v>2.338866286165698E-16</v>
       </c>
       <c r="Q121" s="16">
-        <v>102.3523395</v>
+        <v>46.985986799999999</v>
       </c>
       <c r="R121" s="23">
-        <v>2.2121601319005154E-8</v>
+        <v>1.0093041449742465E-9</v>
       </c>
       <c r="S121" s="23">
-        <v>6.3436970207141882E-11</v>
+        <v>7.5560159000718528E-13</v>
       </c>
     </row>
     <row r="122" spans="1:19" x14ac:dyDescent="0.3">
@@ -7117,49 +7105,49 @@
         <v>6</v>
       </c>
       <c r="B122">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C122">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D122">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E122">
         <v>0</v>
       </c>
       <c r="F122">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G122">
-        <v>864</v>
+        <v>1980</v>
       </c>
       <c r="H122" s="8">
-        <v>7.1990740740740744E-2</v>
+        <v>1.8013468013468013E-2</v>
       </c>
       <c r="I122" s="10">
-        <v>35.144675925925924</v>
+        <v>46.935690235690238</v>
       </c>
       <c r="J122" s="16">
-        <v>1.1869600000000001E-3</v>
+        <v>6.3254666666666673E-3</v>
       </c>
       <c r="K122" s="16">
-        <v>6.5706771599999998</v>
+        <v>16.711406533333331</v>
       </c>
       <c r="L122" s="21">
-        <v>9.1869981011647501E-14</v>
+        <v>2.6698552285433069E-14</v>
       </c>
       <c r="M122" s="21">
-        <v>4.5479560188518037E-16</v>
+        <v>2.378899902841658E-16</v>
       </c>
       <c r="Q122" s="16">
-        <v>5.5931552</v>
+        <v>102.3523395</v>
       </c>
       <c r="R122" s="23">
-        <v>3.6933869379721647E-13</v>
+        <v>2.2121601319005154E-8</v>
       </c>
       <c r="S122" s="23">
-        <v>8.1950857685226958E-15</v>
+        <v>6.3436970207141882E-11</v>
       </c>
     </row>
     <row r="123" spans="1:19" x14ac:dyDescent="0.3">
@@ -7170,96 +7158,96 @@
         <v>3</v>
       </c>
       <c r="C123">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D123">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E123">
         <v>0</v>
       </c>
       <c r="F123">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G123">
-        <v>2160</v>
+        <v>864</v>
       </c>
       <c r="H123" s="8">
-        <v>6.2808641975308638E-2</v>
+        <v>7.1990740740740744E-2</v>
       </c>
       <c r="I123" s="10">
-        <v>36.88148148148148</v>
+        <v>35.144675925925924</v>
       </c>
       <c r="J123" s="16">
-        <v>2.448733333333333E-3</v>
+        <v>1.1869600000000001E-3</v>
       </c>
       <c r="K123" s="16">
-        <v>19.087586566666669</v>
+        <v>6.5706771599999998</v>
       </c>
       <c r="L123" s="21">
-        <v>7.3427908324914067E-14</v>
+        <v>9.1869981011647501E-14</v>
       </c>
       <c r="M123" s="21">
-        <v>4.0285231789900132E-16</v>
+        <v>4.5479560188518037E-16</v>
       </c>
       <c r="Q123" s="16">
-        <v>63.633648000000001</v>
+        <v>5.5931552</v>
       </c>
       <c r="R123" s="23">
-        <v>8.4922962994015287E-12</v>
+        <v>3.6933869379721647E-13</v>
       </c>
       <c r="S123" s="23">
-        <v>1.1454824067240635E-13</v>
+        <v>8.1950857685226958E-15</v>
       </c>
     </row>
     <row r="124" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A124">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B124">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C124">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D124">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E124">
         <v>0</v>
       </c>
       <c r="F124">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G124">
-        <v>147</v>
+        <v>2160</v>
       </c>
       <c r="H124" s="8">
-        <v>5.8503401360544216E-2</v>
+        <v>6.2808641975308638E-2</v>
       </c>
       <c r="I124" s="10">
-        <v>35.657142857142858</v>
+        <v>36.88148148148148</v>
       </c>
       <c r="J124" s="16">
-        <v>5.7081999999999999E-4</v>
+        <v>2.448733333333333E-3</v>
       </c>
       <c r="K124" s="16">
-        <v>0.84981883999999996</v>
+        <v>19.087586566666669</v>
       </c>
       <c r="L124" s="21">
-        <v>4.3767370310090991E-14</v>
+        <v>7.3427908324914067E-14</v>
       </c>
       <c r="M124" s="21">
-        <v>3.6229968385960142E-16</v>
+        <v>4.0285231789900132E-16</v>
       </c>
       <c r="Q124" s="16">
-        <v>0.24576959999999998</v>
+        <v>63.633648000000001</v>
       </c>
       <c r="R124" s="23">
-        <v>4.682050455932844E-13</v>
+        <v>8.4922962994015287E-12</v>
       </c>
       <c r="S124" s="23">
-        <v>6.0345259148311915E-15</v>
+        <v>1.1454824067240635E-13</v>
       </c>
     </row>
     <row r="125" spans="1:19" x14ac:dyDescent="0.3">
@@ -7270,7 +7258,7 @@
         <v>2</v>
       </c>
       <c r="C125">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D125">
         <v>5</v>
@@ -7282,34 +7270,34 @@
         <v>5</v>
       </c>
       <c r="G125">
-        <v>294</v>
+        <v>147</v>
       </c>
       <c r="H125" s="8">
-        <v>3.1292517006802717E-2</v>
+        <v>5.8503401360544216E-2</v>
       </c>
       <c r="I125" s="10">
-        <v>35.801360544217687</v>
+        <v>35.657142857142858</v>
       </c>
       <c r="J125" s="16">
-        <v>9.1216000000000008E-4</v>
+        <v>5.7081999999999999E-4</v>
       </c>
       <c r="K125" s="16">
-        <v>1.4183857999999998</v>
+        <v>0.84981883999999996</v>
       </c>
       <c r="L125" s="21">
-        <v>4.9959691434702983E-14</v>
+        <v>4.3767370310090991E-14</v>
       </c>
       <c r="M125" s="21">
-        <v>3.3077393165211246E-16</v>
+        <v>3.6229968385960142E-16</v>
       </c>
       <c r="Q125" s="16">
-        <v>0.67656028000000001</v>
+        <v>0.24576959999999998</v>
       </c>
       <c r="R125" s="23">
-        <v>1.5703322068510688E-13</v>
+        <v>4.682050455932844E-13</v>
       </c>
       <c r="S125" s="23">
-        <v>5.48789117115168E-15</v>
+        <v>6.0345259148311915E-15</v>
       </c>
     </row>
     <row r="126" spans="1:19" x14ac:dyDescent="0.3">
@@ -7320,7 +7308,7 @@
         <v>2</v>
       </c>
       <c r="C126">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D126">
         <v>5</v>
@@ -7332,34 +7320,34 @@
         <v>5</v>
       </c>
       <c r="G126">
-        <v>490</v>
+        <v>294</v>
       </c>
       <c r="H126" s="8">
-        <v>2.6122448979591838E-2</v>
+        <v>3.1292517006802717E-2</v>
       </c>
       <c r="I126" s="10">
-        <v>37.667755102040815</v>
+        <v>35.801360544217687</v>
       </c>
       <c r="J126" s="16">
-        <v>1.13868E-3</v>
+        <v>9.1216000000000008E-4</v>
       </c>
       <c r="K126" s="16">
-        <v>2.55513536</v>
+        <v>1.4183857999999998</v>
       </c>
       <c r="L126" s="21">
-        <v>4.1938934253409277E-14</v>
+        <v>4.9959691434702983E-14</v>
       </c>
       <c r="M126" s="21">
-        <v>2.9447861754664451E-16</v>
+        <v>3.3077393165211246E-16</v>
       </c>
       <c r="Q126" s="16">
-        <v>1.6750416399999999</v>
+        <v>0.67656028000000001</v>
       </c>
       <c r="R126" s="23">
-        <v>1.000249708918202E-11</v>
+        <v>1.5703322068510688E-13</v>
       </c>
       <c r="S126" s="23">
-        <v>1.9009847282048258E-13</v>
+        <v>5.48789117115168E-15</v>
       </c>
     </row>
     <row r="127" spans="1:19" x14ac:dyDescent="0.3">
@@ -7370,7 +7358,7 @@
         <v>2</v>
       </c>
       <c r="C127">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D127">
         <v>5</v>
@@ -7382,34 +7370,34 @@
         <v>5</v>
       </c>
       <c r="G127">
-        <v>735</v>
+        <v>490</v>
       </c>
       <c r="H127" s="8">
-        <v>1.5238095238095236E-2</v>
+        <v>2.6122448979591838E-2</v>
       </c>
       <c r="I127" s="10">
-        <v>38.644081632653062</v>
+        <v>37.667755102040815</v>
       </c>
       <c r="J127" s="16">
-        <v>1.5916200000000002E-3</v>
+        <v>1.13868E-3</v>
       </c>
       <c r="K127" s="16">
-        <v>4.0244523599999997</v>
+        <v>2.55513536</v>
       </c>
       <c r="L127" s="21">
-        <v>4.7144511320644433E-14</v>
+        <v>4.1938934253409277E-14</v>
       </c>
       <c r="M127" s="21">
-        <v>2.9218715468571781E-16</v>
+        <v>2.9447861754664451E-16</v>
       </c>
       <c r="Q127" s="16">
-        <v>4.4124036600000007</v>
+        <v>1.6750416399999999</v>
       </c>
       <c r="R127" s="23">
-        <v>1.6457575049729394E-11</v>
+        <v>1.000249708918202E-11</v>
       </c>
       <c r="S127" s="23">
-        <v>4.3295340963389813E-14</v>
+        <v>1.9009847282048258E-13</v>
       </c>
     </row>
     <row r="128" spans="1:19" x14ac:dyDescent="0.3">
@@ -7420,7 +7408,7 @@
         <v>2</v>
       </c>
       <c r="C128">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D128">
         <v>5</v>
@@ -7429,37 +7417,37 @@
         <v>0</v>
       </c>
       <c r="F128">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G128">
-        <v>1029</v>
+        <v>735</v>
       </c>
       <c r="H128" s="8">
-        <v>1.6132167152575316E-2</v>
+        <v>1.5238095238095236E-2</v>
       </c>
       <c r="I128" s="10">
-        <v>40.696404275996109</v>
+        <v>38.644081632653062</v>
       </c>
       <c r="J128" s="16">
-        <v>2.3885600000000001E-3</v>
+        <v>1.5916200000000002E-3</v>
       </c>
       <c r="K128" s="16">
-        <v>6.4889960000000002</v>
+        <v>4.0244523599999997</v>
       </c>
       <c r="L128" s="21">
-        <v>4.4763491019978893E-14</v>
+        <v>4.7144511320644433E-14</v>
       </c>
       <c r="M128" s="21">
-        <v>2.8133949240236638E-16</v>
+        <v>2.9218715468571781E-16</v>
       </c>
       <c r="Q128" s="16">
-        <v>11.320121700000001</v>
+        <v>4.4124036600000007</v>
       </c>
       <c r="R128" s="23">
-        <v>7.0330988126507419E-11</v>
+        <v>1.6457575049729394E-11</v>
       </c>
       <c r="S128" s="23">
-        <v>9.3471650781588237E-14</v>
+        <v>4.3295340963389813E-14</v>
       </c>
     </row>
     <row r="129" spans="1:19" x14ac:dyDescent="0.3">
@@ -7470,7 +7458,7 @@
         <v>2</v>
       </c>
       <c r="C129">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D129">
         <v>5</v>
@@ -7482,34 +7470,34 @@
         <v>3</v>
       </c>
       <c r="G129">
-        <v>1372</v>
+        <v>1029</v>
       </c>
       <c r="H129" s="8">
-        <v>1.6763848396501458E-2</v>
+        <v>1.6132167152575316E-2</v>
       </c>
       <c r="I129" s="10">
-        <v>42.527551020408161</v>
+        <v>40.696404275996109</v>
       </c>
       <c r="J129" s="16">
-        <v>3.0201999999999998E-3</v>
+        <v>2.3885600000000001E-3</v>
       </c>
       <c r="K129" s="16">
-        <v>9.5750178399999992</v>
+        <v>6.4889960000000002</v>
       </c>
       <c r="L129" s="21">
-        <v>6.165547267498417E-14</v>
+        <v>4.4763491019978893E-14</v>
       </c>
       <c r="M129" s="21">
-        <v>2.7313915013056855E-16</v>
+        <v>2.8133949240236638E-16</v>
       </c>
       <c r="Q129" s="16">
-        <v>26.342604733333335</v>
+        <v>11.320121700000001</v>
       </c>
       <c r="R129" s="23">
-        <v>1.1004515970393257E-9</v>
+        <v>7.0330988126507419E-11</v>
       </c>
       <c r="S129" s="23">
-        <v>1.7125696000692982E-12</v>
+        <v>9.3471650781588237E-14</v>
       </c>
     </row>
     <row r="130" spans="1:19" x14ac:dyDescent="0.3">
@@ -7520,46 +7508,46 @@
         <v>2</v>
       </c>
       <c r="C130">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D130">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E130">
         <v>0</v>
       </c>
       <c r="F130">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G130">
-        <v>1764</v>
+        <v>1372</v>
       </c>
       <c r="H130" s="8">
-        <v>2.1352985638699924E-2</v>
+        <v>1.6763848396501458E-2</v>
       </c>
       <c r="I130" s="10">
-        <v>44.256046863189717</v>
+        <v>42.527551020408161</v>
       </c>
       <c r="J130" s="16">
-        <v>3.678866666666667E-3</v>
+        <v>3.0201999999999998E-3</v>
       </c>
       <c r="K130" s="16">
-        <v>13.549375533333333</v>
+        <v>9.5750178399999992</v>
       </c>
       <c r="L130" s="21">
-        <v>4.6109730141503417E-14</v>
+        <v>6.165547267498417E-14</v>
       </c>
       <c r="M130" s="21">
-        <v>2.691275822995595E-16</v>
+        <v>2.7313915013056855E-16</v>
       </c>
       <c r="Q130" s="16">
-        <v>61.218966299999998</v>
+        <v>26.342604733333335</v>
       </c>
       <c r="R130" s="23">
-        <v>6.3768511610331396E-9</v>
+        <v>1.1004515970393257E-9</v>
       </c>
       <c r="S130" s="23">
-        <v>1.8693299570517099E-11</v>
+        <v>1.7125696000692982E-12</v>
       </c>
     </row>
     <row r="131" spans="1:19" x14ac:dyDescent="0.3">
@@ -7570,7 +7558,7 @@
         <v>2</v>
       </c>
       <c r="C131">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D131">
         <v>3</v>
@@ -7582,34 +7570,34 @@
         <v>1</v>
       </c>
       <c r="G131">
-        <v>2205</v>
+        <v>1764</v>
       </c>
       <c r="H131" s="8">
-        <v>1.7687074829931974E-2</v>
+        <v>2.1352985638699924E-2</v>
       </c>
       <c r="I131" s="10">
-        <v>45.458956916099773</v>
+        <v>44.256046863189717</v>
       </c>
       <c r="J131" s="16">
-        <v>4.5929999999999999E-3</v>
+        <v>3.678866666666667E-3</v>
       </c>
       <c r="K131" s="16">
-        <v>18.652216299999999</v>
+        <v>13.549375533333333</v>
       </c>
       <c r="L131" s="21">
-        <v>6.9914269748995936E-14</v>
+        <v>4.6109730141503417E-14</v>
       </c>
       <c r="M131" s="21">
-        <v>2.6717841905966925E-16</v>
+        <v>2.691275822995595E-16</v>
       </c>
       <c r="Q131" s="16">
-        <v>148.0203487</v>
+        <v>61.218966299999998</v>
       </c>
       <c r="R131" s="23">
-        <v>6.4137765172045439E-9</v>
+        <v>6.3768511610331396E-9</v>
       </c>
       <c r="S131" s="23">
-        <v>1.2826927984398869E-11</v>
+        <v>1.8693299570517099E-11</v>
       </c>
     </row>
     <row r="132" spans="1:19" x14ac:dyDescent="0.3">
@@ -7620,7 +7608,7 @@
         <v>2</v>
       </c>
       <c r="C132">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D132">
         <v>3</v>
@@ -7632,34 +7620,34 @@
         <v>1</v>
       </c>
       <c r="G132">
-        <v>2695</v>
+        <v>2205</v>
       </c>
       <c r="H132" s="8">
-        <v>1.5089672232529374E-2</v>
+        <v>1.7687074829931974E-2</v>
       </c>
       <c r="I132" s="10">
-        <v>45.776870748299324</v>
+        <v>45.458956916099773</v>
       </c>
       <c r="J132" s="16">
-        <v>5.7049333333333329E-3</v>
+        <v>4.5929999999999999E-3</v>
       </c>
       <c r="K132" s="16">
-        <v>23.026384266666668</v>
+        <v>18.652216299999999</v>
       </c>
       <c r="L132" s="21">
-        <v>4.3380543653820285E-14</v>
+        <v>6.9914269748995936E-14</v>
       </c>
       <c r="M132" s="21">
-        <v>2.6953202427085754E-16</v>
+        <v>2.6717841905966925E-16</v>
       </c>
       <c r="Q132" s="16">
-        <v>205.9769426</v>
+        <v>148.0203487</v>
       </c>
       <c r="R132" s="23">
-        <v>3.5186731033620087E-8</v>
+        <v>6.4137765172045439E-9</v>
       </c>
       <c r="S132" s="23">
-        <v>3.3139170574329736E-11</v>
+        <v>1.2826927984398869E-11</v>
       </c>
     </row>
     <row r="133" spans="1:19" x14ac:dyDescent="0.3">
@@ -7667,10 +7655,10 @@
         <v>7</v>
       </c>
       <c r="B133">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C133">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D133">
         <v>3</v>
@@ -7679,37 +7667,37 @@
         <v>0</v>
       </c>
       <c r="F133">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G133">
-        <v>1372</v>
+        <v>2695</v>
       </c>
       <c r="H133" s="8">
-        <v>9.8882410106899896E-2</v>
+        <v>1.5089672232529374E-2</v>
       </c>
       <c r="I133" s="10">
-        <v>36.218901846452866</v>
+        <v>45.776870748299324</v>
       </c>
       <c r="J133" s="16">
-        <v>1.2840999999999998E-3</v>
+        <v>5.7049333333333329E-3</v>
       </c>
       <c r="K133" s="16">
-        <v>14.6364207</v>
+        <v>23.026384266666668</v>
       </c>
       <c r="L133" s="21">
-        <v>1.642595691875193E-13</v>
+        <v>4.3380543653820285E-14</v>
       </c>
       <c r="M133" s="21">
-        <v>5.3245455941085429E-16</v>
+        <v>2.6953202427085754E-16</v>
       </c>
       <c r="Q133" s="16">
-        <v>17.948652633333335</v>
+        <v>205.9769426</v>
       </c>
       <c r="R133" s="23">
-        <v>2.0200024259194053E-12</v>
+        <v>3.5186731033620087E-8</v>
       </c>
       <c r="S133" s="23">
-        <v>8.7584853768689402E-15</v>
+        <v>3.3139170574329736E-11</v>
       </c>
     </row>
     <row r="134" spans="1:19" x14ac:dyDescent="0.3">
@@ -7720,87 +7708,87 @@
         <v>3</v>
       </c>
       <c r="C134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D134">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E134">
         <v>0</v>
       </c>
       <c r="F134">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G134">
-        <v>3430</v>
+        <v>1372</v>
       </c>
       <c r="H134" s="8">
-        <v>7.1720116618075799E-2</v>
+        <v>9.8882410106899896E-2</v>
       </c>
       <c r="I134" s="10">
-        <v>37.159183673469386</v>
+        <v>36.218901846452866</v>
       </c>
       <c r="J134" s="16">
-        <v>2.7268000000000001E-3</v>
+        <v>1.2840999999999998E-3</v>
       </c>
       <c r="K134" s="16">
-        <v>39.222806599999998</v>
+        <v>14.6364207</v>
       </c>
       <c r="L134" s="21">
-        <v>1.3577917115858543E-13</v>
+        <v>1.642595691875193E-13</v>
       </c>
       <c r="M134" s="21">
-        <v>4.6700913246606915E-16</v>
+        <v>5.3245455941085429E-16</v>
+      </c>
+      <c r="Q134" s="16">
+        <v>17.948652633333335</v>
+      </c>
+      <c r="R134" s="23">
+        <v>2.0200024259194053E-12</v>
+      </c>
+      <c r="S134" s="23">
+        <v>8.7584853768689402E-15</v>
       </c>
     </row>
     <row r="135" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A135">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B135">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C135">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D135">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E135">
         <v>0</v>
       </c>
       <c r="F135">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G135">
-        <v>300</v>
-      </c>
-      <c r="H135" s="49">
-        <v>6.13E-2</v>
-      </c>
-      <c r="I135" s="50">
-        <v>34.5</v>
-      </c>
-      <c r="J135" s="51">
-        <v>7.4599999999999996E-3</v>
-      </c>
-      <c r="K135" s="51">
-        <v>2.375</v>
-      </c>
-      <c r="L135" s="52">
-        <v>1.2999999999999999E-12</v>
-      </c>
-      <c r="M135" s="52">
-        <v>5.34E-16</v>
-      </c>
-      <c r="Q135" s="16">
-        <v>0.88176655999999998</v>
-      </c>
-      <c r="R135" s="23">
-        <v>6.1198168891026161E-13</v>
-      </c>
-      <c r="S135" s="23">
-        <v>9.4429430014736385E-15</v>
+        <v>3430</v>
+      </c>
+      <c r="H135" s="8">
+        <v>7.1720116618075799E-2</v>
+      </c>
+      <c r="I135" s="10">
+        <v>37.159183673469386</v>
+      </c>
+      <c r="J135" s="16">
+        <v>2.7268000000000001E-3</v>
+      </c>
+      <c r="K135" s="16">
+        <v>39.222806599999998</v>
+      </c>
+      <c r="L135" s="21">
+        <v>1.3577917115858543E-13</v>
+      </c>
+      <c r="M135" s="21">
+        <v>4.6700913246606915E-16</v>
       </c>
     </row>
     <row r="136" spans="1:19" x14ac:dyDescent="0.3">
@@ -7811,7 +7799,7 @@
         <v>2</v>
       </c>
       <c r="C136">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D136">
         <v>5</v>
@@ -7823,34 +7811,34 @@
         <v>5</v>
       </c>
       <c r="G136">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="H136" s="49">
-        <v>4.36E-2</v>
+        <v>6.13E-2</v>
       </c>
       <c r="I136" s="50">
-        <v>36.137999999999998</v>
+        <v>34.5</v>
       </c>
       <c r="J136" s="51">
-        <v>2.0000000000000001E-4</v>
+        <v>7.4599999999999996E-3</v>
       </c>
       <c r="K136" s="51">
-        <v>3.9319000000000002</v>
+        <v>2.375</v>
       </c>
       <c r="L136" s="52">
-        <v>2.4199999999999998E-13</v>
+        <v>1.2999999999999999E-12</v>
       </c>
       <c r="M136" s="52">
-        <v>4.5899999999999996E-16</v>
+        <v>5.34E-16</v>
       </c>
       <c r="Q136" s="16">
-        <v>2.8232591999999999</v>
+        <v>0.88176655999999998</v>
       </c>
       <c r="R136" s="23">
-        <v>5.0217809093392962E-12</v>
+        <v>6.1198168891026161E-13</v>
       </c>
       <c r="S136" s="23">
-        <v>5.9206065875100495E-14</v>
+        <v>9.4429430014736385E-15</v>
       </c>
     </row>
     <row r="137" spans="1:19" x14ac:dyDescent="0.3">
@@ -7861,7 +7849,7 @@
         <v>2</v>
       </c>
       <c r="C137">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D137">
         <v>5</v>
@@ -7873,34 +7861,34 @@
         <v>5</v>
       </c>
       <c r="G137">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="H137" s="49">
-        <v>3.7199999999999997E-2</v>
+        <v>4.36E-2</v>
       </c>
       <c r="I137" s="50">
-        <v>37.22</v>
+        <v>36.137999999999998</v>
       </c>
       <c r="J137" s="51">
-        <v>1E-3</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="K137" s="51">
-        <v>6.31</v>
+        <v>3.9319000000000002</v>
       </c>
       <c r="L137" s="52">
-        <v>2.37E-13</v>
+        <v>2.4199999999999998E-13</v>
       </c>
       <c r="M137" s="52">
-        <v>4.2600000000000002E-16</v>
+        <v>4.5899999999999996E-16</v>
       </c>
       <c r="Q137" s="16">
-        <v>9.4948389399999993</v>
+        <v>2.8232591999999999</v>
       </c>
       <c r="R137" s="23">
-        <v>5.4344423379448989E-12</v>
+        <v>5.0217809093392962E-12</v>
       </c>
       <c r="S137" s="23">
-        <v>2.6273268378747125E-14</v>
+        <v>5.9206065875100495E-14</v>
       </c>
     </row>
     <row r="138" spans="1:19" x14ac:dyDescent="0.3">
@@ -7911,46 +7899,46 @@
         <v>2</v>
       </c>
       <c r="C138">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D138">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E138">
         <v>0</v>
       </c>
       <c r="F138">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G138">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="H138" s="49">
-        <v>2.0400000000000001E-2</v>
+        <v>3.7199999999999997E-2</v>
       </c>
       <c r="I138" s="50">
-        <v>38.636000000000003</v>
+        <v>37.22</v>
       </c>
       <c r="J138" s="51">
-        <v>1.8703333333333332E-3</v>
+        <v>1E-3</v>
       </c>
       <c r="K138" s="51">
-        <v>10.183</v>
+        <v>6.31</v>
       </c>
       <c r="L138" s="52">
-        <v>2.41E-14</v>
+        <v>2.37E-13</v>
       </c>
       <c r="M138" s="52">
-        <v>4.0599999999999999E-16</v>
+        <v>4.2600000000000002E-16</v>
       </c>
       <c r="Q138" s="16">
-        <v>31.7727264</v>
+        <v>9.4948389399999993</v>
       </c>
       <c r="R138" s="23">
-        <v>1.0818483964618036E-11</v>
+        <v>5.4344423379448989E-12</v>
       </c>
       <c r="S138" s="23">
-        <v>4.5887318376204904E-14</v>
+        <v>2.6273268378747125E-14</v>
       </c>
     </row>
     <row r="139" spans="1:19" x14ac:dyDescent="0.3">
@@ -7961,7 +7949,7 @@
         <v>2</v>
       </c>
       <c r="C139">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D139">
         <v>3</v>
@@ -7973,144 +7961,194 @@
         <v>1</v>
       </c>
       <c r="G139">
+        <v>1500</v>
+      </c>
+      <c r="H139" s="49">
+        <v>2.0400000000000001E-2</v>
+      </c>
+      <c r="I139" s="50">
+        <v>38.636000000000003</v>
+      </c>
+      <c r="J139" s="51">
+        <v>1.8703333333333332E-3</v>
+      </c>
+      <c r="K139" s="51">
+        <v>10.183</v>
+      </c>
+      <c r="L139" s="52">
+        <v>2.41E-14</v>
+      </c>
+      <c r="M139" s="52">
+        <v>4.0599999999999999E-16</v>
+      </c>
+      <c r="Q139" s="16">
+        <v>31.7727264</v>
+      </c>
+      <c r="R139" s="23">
+        <v>1.0818483964618036E-11</v>
+      </c>
+      <c r="S139" s="23">
+        <v>4.5887318376204904E-14</v>
+      </c>
+    </row>
+    <row r="140" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A140">
+        <v>10</v>
+      </c>
+      <c r="B140">
+        <v>2</v>
+      </c>
+      <c r="C140">
+        <v>6</v>
+      </c>
+      <c r="D140">
+        <v>3</v>
+      </c>
+      <c r="E140">
+        <v>0</v>
+      </c>
+      <c r="F140">
+        <v>1</v>
+      </c>
+      <c r="G140">
         <v>2100</v>
       </c>
-      <c r="H139" s="49">
+      <c r="H140" s="49">
         <v>2.41E-2</v>
       </c>
-      <c r="I139" s="50">
+      <c r="I140" s="50">
         <v>40.487000000000002</v>
       </c>
-      <c r="J139" s="51">
+      <c r="J140" s="51">
         <v>2.7100000000000002E-3</v>
       </c>
-      <c r="K139" s="51">
+      <c r="K140" s="51">
         <v>16.943999999999999</v>
       </c>
-      <c r="L139" s="52">
+      <c r="L140" s="52">
         <v>2.5900000000000001E-13</v>
       </c>
-      <c r="M139" s="52">
+      <c r="M140" s="52">
         <v>3.954135446458232E-16</v>
       </c>
-      <c r="Q139" s="16">
+      <c r="Q140" s="16">
         <v>105.6478079</v>
       </c>
-      <c r="R139" s="23">
+      <c r="R140" s="23">
         <v>3.549609196044045E-9</v>
       </c>
-      <c r="S139" s="23">
+      <c r="S140" s="23">
         <v>2.5864833288222837E-12</v>
       </c>
     </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A140" s="12">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A141" s="12">
         <v>15</v>
       </c>
-      <c r="B140" s="12">
-        <v>2</v>
-      </c>
-      <c r="C140" s="12">
-        <v>2</v>
-      </c>
-      <c r="D140" s="12">
-        <v>5</v>
-      </c>
-      <c r="E140" s="12">
-        <v>0</v>
-      </c>
-      <c r="F140" s="12">
-        <v>5</v>
-      </c>
-      <c r="G140" s="12">
+      <c r="B141" s="12">
+        <v>2</v>
+      </c>
+      <c r="C141" s="12">
+        <v>2</v>
+      </c>
+      <c r="D141" s="12">
+        <v>5</v>
+      </c>
+      <c r="E141" s="12">
+        <v>0</v>
+      </c>
+      <c r="F141" s="12">
+        <v>5</v>
+      </c>
+      <c r="G141" s="12">
         <v>675</v>
       </c>
-      <c r="H140" s="13">
+      <c r="H141" s="13">
         <v>5.8900000000000001E-2</v>
       </c>
-      <c r="I140" s="14">
+      <c r="I141" s="14">
         <v>34.292000000000002</v>
       </c>
-      <c r="J140" s="17">
+      <c r="J141" s="17">
         <v>6.7227999999999993E-4</v>
       </c>
-      <c r="K140" s="17">
+      <c r="K141" s="17">
         <v>5.9416000000000002</v>
       </c>
-      <c r="L140" s="22">
+      <c r="L141" s="22">
         <v>0.17199566509229403</v>
       </c>
-      <c r="M140" s="22">
+      <c r="M141" s="22">
         <v>8.7618527618346915E-16</v>
       </c>
-      <c r="N140" s="17"/>
-      <c r="O140" s="24"/>
-      <c r="P140" s="24"/>
-      <c r="Q140" s="17">
+      <c r="N141" s="17"/>
+      <c r="O141" s="24"/>
+      <c r="P141" s="24"/>
+      <c r="Q141" s="17">
         <v>4.5755377399999997</v>
       </c>
-      <c r="R140" s="24">
+      <c r="R141" s="24">
         <v>6.2632535913292558E-12</v>
       </c>
-      <c r="S140" s="24">
+      <c r="S141" s="24">
         <v>1.6035885772533078E-13</v>
       </c>
     </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A141">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A142">
         <v>20</v>
       </c>
-      <c r="B141">
-        <v>2</v>
-      </c>
-      <c r="C141">
-        <v>2</v>
-      </c>
-      <c r="D141">
-        <v>3</v>
-      </c>
-      <c r="E141">
-        <v>0</v>
-      </c>
-      <c r="F141">
-        <v>3</v>
-      </c>
-      <c r="G141">
+      <c r="B142">
+        <v>2</v>
+      </c>
+      <c r="C142">
+        <v>2</v>
+      </c>
+      <c r="D142">
+        <v>3</v>
+      </c>
+      <c r="E142">
+        <v>0</v>
+      </c>
+      <c r="F142">
+        <v>3</v>
+      </c>
+      <c r="G142">
         <v>1200</v>
       </c>
-      <c r="H141" s="49">
+      <c r="H142" s="49">
         <v>8.1100000000000005E-2</v>
       </c>
-      <c r="I141" s="50">
+      <c r="I142" s="50">
         <v>35.186999999999998</v>
       </c>
-      <c r="J141" s="51">
+      <c r="J142" s="51">
         <v>7.9946666666666673E-4</v>
       </c>
-      <c r="K141" s="51">
+      <c r="K142" s="51">
         <v>16.3</v>
       </c>
-      <c r="L141" s="52">
+      <c r="L142" s="52">
         <v>8.84E-11</v>
       </c>
-      <c r="M141" s="52">
+      <c r="M142" s="52">
         <v>3.5399999999999999E-15</v>
       </c>
-      <c r="Q141" s="16">
+      <c r="Q142" s="16">
         <v>18.132396066666669</v>
       </c>
-      <c r="R141" s="23">
+      <c r="R142" s="23">
         <v>1.1242075415885675E-12</v>
       </c>
-      <c r="S141" s="23">
+      <c r="S142" s="23">
         <v>3.4699449019803669E-14</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:X141">
-    <sortCondition ref="A2:A141"/>
-    <sortCondition ref="B2:B141"/>
-    <sortCondition ref="C2:C141"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:X142">
+    <sortCondition ref="A2:A142"/>
+    <sortCondition ref="B2:B142"/>
+    <sortCondition ref="C2:C142"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>